<commit_message>
docs: add project work plan
</commit_message>
<xml_diff>
--- a/docs/Arbets-struktur/Utförande.xlsx
+++ b/docs/Arbets-struktur/Utförande.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="80">
   <si>
     <t>Fas</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Databas &amp; Backend</t>
   </si>
   <si>
-    <t>Etablerade anslutning till databasen (feature/db-connection).</t>
-  </si>
-  <si>
     <t>Admin &amp; Kontrollpanel</t>
   </si>
   <si>
@@ -151,7 +148,109 @@
     <t>ANDREAS:</t>
   </si>
   <si>
+    <t xml:space="preserve">14 sep – 17 sep </t>
+  </si>
+  <si>
+    <t>Planering &amp; DB-koppling</t>
+  </si>
+  <si>
+    <t>Deltog i projektplanering och etablerade anslutning till databasen (feature/db-connection).</t>
+  </si>
+  <si>
+    <t>Pricing &amp; Courses</t>
+  </si>
+  <si>
+    <t>Implementerade Pricing- och Courses-sidorna samt navigation mellan sidor.</t>
+  </si>
+  <si>
+    <t>14 sep - 17 sep</t>
+  </si>
+  <si>
+    <t>Datainmatning</t>
+  </si>
+  <si>
+    <t>Fyllde databasen med kurs-, lektions- och quizdata för att kunna testa och använda funktionerna i applikationen.</t>
+  </si>
+  <si>
+    <t>Fas 2: Funktionalitet &amp; Autentisering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 sep – 22 sep </t>
+  </si>
+  <si>
+    <t>CoursePage &amp; Lessons</t>
+  </si>
+  <si>
+    <t>Implementerade CoursePage och visning av lektioner från API:t.</t>
+  </si>
+  <si>
+    <t>Payment &amp; Authentication</t>
+  </si>
+  <si>
+    <t>Implementerade checkout-flöde och autentisering med JWT-token i API-anrop.</t>
+  </si>
+  <si>
+    <t>Loading &amp; Error states</t>
+  </si>
+  <si>
+    <t>Lade till loading states, felhantering och användarmeddelanden.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 sep – 24 sep </t>
+  </si>
+  <si>
+    <t>LessonPage &amp; QuizPage</t>
+  </si>
+  <si>
+    <t>Implementerade LessonPage och QuizPage med innehåll, frågor och svar.</t>
+  </si>
+  <si>
+    <t>Fas 3: Åtkomstkontroll &amp; UX</t>
+  </si>
+  <si>
+    <t>24 sep - 30 sep</t>
+  </si>
+  <si>
+    <t>Quiz &amp; Access Control</t>
+  </si>
+  <si>
+    <t>Utvecklade quizfunktionalitet och behörighetskontroll baserat på abonnemangsnivå.</t>
+  </si>
+  <si>
+    <t>Responsive design &amp; UX</t>
+  </si>
+  <si>
+    <t>Förbättrade responsiv design, användarupplevelse och navigation samt använde semantiskt HTML.</t>
+  </si>
+  <si>
+    <t>Fas 4: Funktionalitet, Refaktorering &amp; Responsive Design</t>
+  </si>
+  <si>
+    <t>1 okt</t>
+  </si>
+  <si>
+    <t>Refaktorering &amp; komponentstruktur</t>
+  </si>
+  <si>
+    <t>Refaktorerade komponenter och skapade återanvändbara list- och knappkomponenter.</t>
+  </si>
+  <si>
+    <t>CheckoutPage</t>
+  </si>
+  <si>
+    <t>Implementerade CheckoutPage för att hantera användarens val av abonnemang och genomföra checkout-flödet mot backend.</t>
+  </si>
+  <si>
+    <t>Responsive design</t>
+  </si>
+  <si>
+    <t>Anpassade webbplatsens layout och komponenter för mobil och mindre skärmar.</t>
+  </si>
+  <si>
     <t>WILLIAM:</t>
+  </si>
+  <si>
+    <t>§</t>
   </si>
 </sst>
 </file>
@@ -495,9 +594,7 @@
       <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>10</v>
-      </c>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -507,10 +604,10 @@
         <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -521,242 +618,338 @@
         <v>6</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="C8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="C9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="C11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>30</v>
-      </c>
       <c r="C13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>30</v>
-      </c>
       <c r="C14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>38</v>
-      </c>
       <c r="C16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>38</v>
-      </c>
       <c r="C17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
+      <c r="C20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
+      <c r="A21" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
+      <c r="A22" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
+      <c r="A23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
+      <c r="A24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
+      <c r="A25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
+      <c r="A26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
+      <c r="A27" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
+      <c r="A28" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
+      <c r="A29" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
+      <c r="A30" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
+      <c r="A31" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
@@ -787,10 +980,14 @@
     <row r="38" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="40" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>79</v>
+      </c>
+    </row>
     <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="43" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>